<commit_message>
Homogenized cursor placement and zoom between Excel sheets
</commit_message>
<xml_diff>
--- a/data/20251212-OdonTraits_Europe.xlsx
+++ b/data/20251212-OdonTraits_Europe.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1680" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="6"/>
+    <workbookView xWindow="28680" yWindow="1680" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="taxonomic" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">protection_endemism!$A$1:$G$144</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">taxonomic!$A$1:$E$144</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -11479,11 +11479,11 @@
         <v>68</v>
       </c>
       <c r="B22" s="8">
-        <f t="shared" ref="B22:C25" si="0">D22+F22</f>
+        <f>D22+F22</f>
         <v>28</v>
       </c>
       <c r="C22" s="8">
-        <f t="shared" si="0"/>
+        <f>E22+G22</f>
         <v>31</v>
       </c>
       <c r="D22" s="8">
@@ -11504,11 +11504,11 @@
         <v>73</v>
       </c>
       <c r="B23" s="8">
-        <f t="shared" si="0"/>
+        <f>D23+F23</f>
         <v>27</v>
       </c>
       <c r="C23" s="8">
-        <f t="shared" si="0"/>
+        <f>E23+G23</f>
         <v>38</v>
       </c>
       <c r="D23" s="8">
@@ -11529,11 +11529,11 @@
         <v>76</v>
       </c>
       <c r="B24" s="8">
-        <f t="shared" si="0"/>
+        <f>D24+F24</f>
         <v>23</v>
       </c>
       <c r="C24" s="8">
-        <f t="shared" si="0"/>
+        <f>E24+G24</f>
         <v>34</v>
       </c>
       <c r="D24" s="8">
@@ -11554,11 +11554,11 @@
         <v>79</v>
       </c>
       <c r="B25" s="8">
-        <f t="shared" si="0"/>
+        <f>D25+F25</f>
         <v>31</v>
       </c>
       <c r="C25" s="8">
-        <f t="shared" si="0"/>
+        <f>E25+G25</f>
         <v>36</v>
       </c>
       <c r="D25" s="8">
@@ -11602,11 +11602,11 @@
         <v>87</v>
       </c>
       <c r="B27" s="8">
-        <f t="shared" ref="B27:C32" si="1">D27+F27</f>
+        <f>D27+F27</f>
         <v>15</v>
       </c>
       <c r="C27" s="8">
-        <f t="shared" si="1"/>
+        <f>E27+G27</f>
         <v>19</v>
       </c>
       <c r="D27" s="8">
@@ -11627,11 +11627,11 @@
         <v>299</v>
       </c>
       <c r="B28" s="8">
-        <f t="shared" si="1"/>
+        <f>D28+F28</f>
         <v>23</v>
       </c>
       <c r="C28" s="8">
-        <f t="shared" si="1"/>
+        <f>E28+G28</f>
         <v>29</v>
       </c>
       <c r="D28" s="8">
@@ -11652,11 +11652,11 @@
         <v>304</v>
       </c>
       <c r="B29" s="8">
-        <f t="shared" si="1"/>
+        <f>D29+F29</f>
         <v>23</v>
       </c>
       <c r="C29" s="8">
-        <f t="shared" si="1"/>
+        <f>E29+G29</f>
         <v>29</v>
       </c>
       <c r="D29" s="8">
@@ -11677,11 +11677,11 @@
         <v>90</v>
       </c>
       <c r="B30" s="8">
-        <f t="shared" si="1"/>
+        <f>D30+F30</f>
         <v>19</v>
       </c>
       <c r="C30" s="8">
-        <f t="shared" si="1"/>
+        <f>E30+G30</f>
         <v>23</v>
       </c>
       <c r="D30" s="8">
@@ -11702,11 +11702,11 @@
         <v>94</v>
       </c>
       <c r="B31" s="8">
-        <f t="shared" si="1"/>
+        <f>D31+F31</f>
         <v>14</v>
       </c>
       <c r="C31" s="8">
-        <f t="shared" si="1"/>
+        <f>E31+G31</f>
         <v>18</v>
       </c>
       <c r="D31" s="8">
@@ -11727,11 +11727,11 @@
         <v>517</v>
       </c>
       <c r="B32" s="8">
-        <f t="shared" si="1"/>
+        <f>D32+F32</f>
         <v>14</v>
       </c>
       <c r="C32" s="8">
-        <f t="shared" si="1"/>
+        <f>E32+G32</f>
         <v>18</v>
       </c>
       <c r="D32" s="8">
@@ -11798,11 +11798,11 @@
         <v>106</v>
       </c>
       <c r="B35" s="8">
-        <f t="shared" ref="B35:B44" si="2">D35+F35</f>
+        <f>D35+F35</f>
         <v>20</v>
       </c>
       <c r="C35" s="8">
-        <f t="shared" ref="C35:C44" si="3">E35+G35</f>
+        <f>E35+G35</f>
         <v>23</v>
       </c>
       <c r="D35" s="8">
@@ -11823,11 +11823,11 @@
         <v>109</v>
       </c>
       <c r="B36" s="8">
-        <f t="shared" si="2"/>
+        <f>D36+F36</f>
         <v>21</v>
       </c>
       <c r="C36" s="8">
-        <f t="shared" si="3"/>
+        <f>E36+G36</f>
         <v>23</v>
       </c>
       <c r="D36" s="8">
@@ -11848,11 +11848,11 @@
         <v>112</v>
       </c>
       <c r="B37" s="8">
-        <f t="shared" si="2"/>
+        <f>D37+F37</f>
         <v>18</v>
       </c>
       <c r="C37" s="8">
-        <f t="shared" si="3"/>
+        <f>E37+G37</f>
         <v>21</v>
       </c>
       <c r="D37" s="8">
@@ -11873,11 +11873,11 @@
         <v>115</v>
       </c>
       <c r="B38" s="8">
-        <f t="shared" si="2"/>
+        <f>D38+F38</f>
         <v>13</v>
       </c>
       <c r="C38" s="8">
-        <f t="shared" si="3"/>
+        <f>E38+G38</f>
         <v>14.5</v>
       </c>
       <c r="D38" s="8">
@@ -11898,11 +11898,11 @@
         <v>118</v>
       </c>
       <c r="B39" s="8">
-        <f t="shared" si="2"/>
+        <f>D39+F39</f>
         <v>19</v>
       </c>
       <c r="C39" s="8">
-        <f t="shared" si="3"/>
+        <f>E39+G39</f>
         <v>25</v>
       </c>
       <c r="D39" s="8">
@@ -11923,11 +11923,11 @@
         <v>121</v>
       </c>
       <c r="B40" s="8">
-        <f t="shared" si="2"/>
+        <f>D40+F40</f>
         <v>14</v>
       </c>
       <c r="C40" s="8">
-        <f t="shared" si="3"/>
+        <f>E40+G40</f>
         <v>18</v>
       </c>
       <c r="D40" s="8">
@@ -11948,11 +11948,11 @@
         <v>124</v>
       </c>
       <c r="B41" s="8">
-        <f t="shared" si="2"/>
+        <f>D41+F41</f>
         <v>15</v>
       </c>
       <c r="C41" s="8">
-        <f t="shared" si="3"/>
+        <f>E41+G41</f>
         <v>19</v>
       </c>
       <c r="D41" s="8">
@@ -11973,11 +11973,11 @@
         <v>127</v>
       </c>
       <c r="B42" s="8">
-        <f t="shared" si="2"/>
+        <f>D42+F42</f>
         <v>17</v>
       </c>
       <c r="C42" s="8">
-        <f t="shared" si="3"/>
+        <f>E42+G42</f>
         <v>21</v>
       </c>
       <c r="D42" s="8">
@@ -11998,11 +11998,11 @@
         <v>130</v>
       </c>
       <c r="B43" s="8">
-        <f t="shared" si="2"/>
+        <f>D43+F43</f>
         <v>17</v>
       </c>
       <c r="C43" s="8">
-        <f t="shared" si="3"/>
+        <f>E43+G43</f>
         <v>20</v>
       </c>
       <c r="D43" s="8">
@@ -12023,11 +12023,11 @@
         <v>133</v>
       </c>
       <c r="B44" s="8">
-        <f t="shared" si="2"/>
+        <f>D44+F44</f>
         <v>14</v>
       </c>
       <c r="C44" s="8">
-        <f t="shared" si="3"/>
+        <f>E44+G44</f>
         <v>21</v>
       </c>
       <c r="D44" s="8">
@@ -12351,11 +12351,11 @@
         <v>140</v>
       </c>
       <c r="B58" s="8">
-        <f t="shared" ref="B58:C60" si="4">D58+F58</f>
+        <f>D58+F58</f>
         <v>18</v>
       </c>
       <c r="C58" s="8">
-        <f t="shared" si="4"/>
+        <f>E58+G58</f>
         <v>22</v>
       </c>
       <c r="D58" s="8">
@@ -12376,11 +12376,11 @@
         <v>144</v>
       </c>
       <c r="B59" s="8">
-        <f t="shared" si="4"/>
+        <f>D59+F59</f>
         <v>25</v>
       </c>
       <c r="C59" s="8">
-        <f t="shared" si="4"/>
+        <f>E59+G59</f>
         <v>31</v>
       </c>
       <c r="D59" s="8">
@@ -12401,11 +12401,11 @@
         <v>147</v>
       </c>
       <c r="B60" s="8">
-        <f t="shared" si="4"/>
+        <f>D60+F60</f>
         <v>17</v>
       </c>
       <c r="C60" s="8">
-        <f t="shared" si="4"/>
+        <f>E60+G60</f>
         <v>20</v>
       </c>
       <c r="D60" s="8">
@@ -12564,11 +12564,11 @@
         <v>154</v>
       </c>
       <c r="B67" s="8">
-        <f t="shared" ref="B67:C70" si="5">D67+F67</f>
+        <f>D67+F67</f>
         <v>18</v>
       </c>
       <c r="C67" s="8">
-        <f t="shared" si="5"/>
+        <f>E67+G67</f>
         <v>21</v>
       </c>
       <c r="D67" s="8">
@@ -12589,11 +12589,11 @@
         <v>157</v>
       </c>
       <c r="B68" s="8">
-        <f t="shared" si="5"/>
+        <f>D68+F68</f>
         <v>17</v>
       </c>
       <c r="C68" s="8">
-        <f t="shared" si="5"/>
+        <f>E68+G68</f>
         <v>21</v>
       </c>
       <c r="D68" s="8">
@@ -12614,11 +12614,11 @@
         <v>160</v>
       </c>
       <c r="B69" s="8">
-        <f t="shared" si="5"/>
+        <f>D69+F69</f>
         <v>16</v>
       </c>
       <c r="C69" s="8">
-        <f t="shared" si="5"/>
+        <f>E69+G69</f>
         <v>21</v>
       </c>
       <c r="D69" s="8">
@@ -12639,11 +12639,11 @@
         <v>163</v>
       </c>
       <c r="B70" s="8">
-        <f t="shared" si="5"/>
+        <f>D70+F70</f>
         <v>16</v>
       </c>
       <c r="C70" s="8">
-        <f t="shared" si="5"/>
+        <f>E70+G70</f>
         <v>19</v>
       </c>
       <c r="D70" s="8">
@@ -12781,11 +12781,11 @@
         <v>306</v>
       </c>
       <c r="B76" s="8">
-        <f t="shared" ref="B76:C80" si="6">D76+F76</f>
+        <f>D76+F76</f>
         <v>23</v>
       </c>
       <c r="C76" s="8">
-        <f t="shared" si="6"/>
+        <f>E76+G76</f>
         <v>26</v>
       </c>
       <c r="D76" s="8">
@@ -12806,11 +12806,11 @@
         <v>310</v>
       </c>
       <c r="B77" s="8">
-        <f t="shared" si="6"/>
+        <f>D77+F77</f>
         <v>24</v>
       </c>
       <c r="C77" s="8">
-        <f t="shared" si="6"/>
+        <f>E77+G77</f>
         <v>35</v>
       </c>
       <c r="D77" s="8">
@@ -12831,11 +12831,11 @@
         <v>313</v>
       </c>
       <c r="B78" s="8">
-        <f t="shared" si="6"/>
+        <f>D78+F78</f>
         <v>22</v>
       </c>
       <c r="C78" s="8">
-        <f t="shared" si="6"/>
+        <f>E78+G78</f>
         <v>29</v>
       </c>
       <c r="D78" s="8">
@@ -12856,11 +12856,11 @@
         <v>316</v>
       </c>
       <c r="B79" s="8">
-        <f t="shared" si="6"/>
+        <f>D79+F79</f>
         <v>24</v>
       </c>
       <c r="C79" s="8">
-        <f t="shared" si="6"/>
+        <f>E79+G79</f>
         <v>31</v>
       </c>
       <c r="D79" s="8">
@@ -12881,11 +12881,11 @@
         <v>319</v>
       </c>
       <c r="B80" s="8">
-        <f t="shared" si="6"/>
+        <f>D80+F80</f>
         <v>22</v>
       </c>
       <c r="C80" s="8">
-        <f t="shared" si="6"/>
+        <f>E80+G80</f>
         <v>26</v>
       </c>
       <c r="D80" s="8">
@@ -13598,11 +13598,11 @@
         <v>465</v>
       </c>
       <c r="B111" s="8">
-        <f t="shared" ref="B111:C113" si="7">D111+F111</f>
+        <f>D111+F111</f>
         <v>18</v>
       </c>
       <c r="C111" s="8">
-        <f t="shared" si="7"/>
+        <f>E111+G111</f>
         <v>22</v>
       </c>
       <c r="D111" s="8">
@@ -13623,11 +13623,11 @@
         <v>470</v>
       </c>
       <c r="B112" s="8">
-        <f t="shared" si="7"/>
+        <f>D112+F112</f>
         <v>16</v>
       </c>
       <c r="C112" s="8">
-        <f t="shared" si="7"/>
+        <f>E112+G112</f>
         <v>19</v>
       </c>
       <c r="D112" s="8">
@@ -13648,11 +13648,11 @@
         <v>473</v>
       </c>
       <c r="B113" s="8">
-        <f t="shared" si="7"/>
+        <f>D113+F113</f>
         <v>18</v>
       </c>
       <c r="C113" s="8">
-        <f t="shared" si="7"/>
+        <f>E113+G113</f>
         <v>24</v>
       </c>
       <c r="D113" s="8">

</xml_diff>